<commit_message>
Update Extended Data Fig. 5 workbook and panel statistics documentation
</commit_message>
<xml_diff>
--- a/experiments_revision/matched_sequence_circulation/plotting_reference/Extended_Data_Fig_5_Plot_Data.xlsx
+++ b/experiments_revision/matched_sequence_circulation/plotting_reference/Extended_Data_Fig_5_Plot_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowHeight="17680" activeTab="3"/>
+    <workbookView windowWidth="24750" windowHeight="10480" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="a Substitutions" sheetId="1" r:id="rId1"/>
@@ -1433,27 +1433,27 @@
         <v>13</v>
       </c>
       <c r="C6" s="13">
-        <v>99.27</v>
+        <v>99.3</v>
       </c>
       <c r="D6" s="13">
-        <v>99.86</v>
+        <v>99.9</v>
       </c>
       <c r="E6" s="13">
-        <v>99.93</v>
+        <v>99.9</v>
       </c>
       <c r="F6" s="13">
-        <v>99.95</v>
+        <v>100</v>
       </c>
       <c r="G6" s="13">
-        <v>99.99</v>
+        <v>100</v>
       </c>
       <c r="H6" s="14">
         <f t="shared" si="0"/>
-        <v>99.8</v>
+        <v>99.82</v>
       </c>
       <c r="I6" s="14">
         <f t="shared" si="1"/>
-        <v>0.300000000000002</v>
+        <v>0.294957624075055</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" spans="1:9">
@@ -2001,27 +2001,27 @@
         <v>13</v>
       </c>
       <c r="C6" s="13">
-        <v>99.27</v>
+        <v>99.3</v>
       </c>
       <c r="D6" s="13">
-        <v>99.86</v>
+        <v>99.8</v>
       </c>
       <c r="E6" s="13">
-        <v>99.93</v>
+        <v>99.9</v>
       </c>
       <c r="F6" s="13">
-        <v>99.95</v>
+        <v>99.9</v>
       </c>
       <c r="G6" s="13">
-        <v>99.99</v>
+        <v>100</v>
       </c>
       <c r="H6" s="14">
         <f t="shared" si="0"/>
-        <v>99.8</v>
+        <v>99.78</v>
       </c>
       <c r="I6" s="14">
         <f t="shared" si="1"/>
-        <v>0.300000000000002</v>
+        <v>0.277488738510235</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" spans="1:9">
@@ -2569,27 +2569,27 @@
         <v>13</v>
       </c>
       <c r="C6" s="13">
-        <v>99.27</v>
+        <v>99.3</v>
       </c>
       <c r="D6" s="13">
-        <v>99.86</v>
+        <v>99.8</v>
       </c>
       <c r="E6" s="13">
-        <v>99.93</v>
+        <v>99.9</v>
       </c>
       <c r="F6" s="13">
-        <v>99.95</v>
+        <v>99.9</v>
       </c>
       <c r="G6" s="13">
-        <v>99.99</v>
+        <v>100</v>
       </c>
       <c r="H6" s="14">
         <f t="shared" si="0"/>
-        <v>99.8</v>
+        <v>99.78</v>
       </c>
       <c r="I6" s="14">
         <f t="shared" si="1"/>
-        <v>0.300000000000002</v>
+        <v>0.277488738510235</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" spans="1:9">

</xml_diff>